<commit_message>
changed fixures for eu taxo financials 2026 and updated the input xlsx for eu taxo non financials 2026
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d20024\Documents\proj1_d50_Dataland\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93795\Desktop\dataland\dataland\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF251514-3A78-44E4-8EF4-B10B1EA98E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B95AF64-5C72-42D3-85B6-557E17CEFDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26550" yWindow="1425" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="168">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -502,126 +502,6 @@
     <t>Relative share of the OpEx that is associated with economic activities that are considered non-material with respect to the OpEx and not assessed for Taxonomy-eligibility and Taxonomy-alignment in accordance with Article 2(1a), (1b), and (1c) of Regulation (EU) 2026/73, respectively</t>
   </si>
   <si>
-    <t>13.1</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>13.2</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>26.1</t>
-  </si>
-  <si>
-    <t>26.2</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>39.1</t>
-  </si>
-  <si>
-    <t>39.2</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>49</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
     <t>Eligible or Aligned Activities</t>
   </si>
   <si>
@@ -629,9 +509,6 @@
   </si>
   <si>
     <t>Custom EuTaxonomyEligibleOrAlignedActivitiesComponent</t>
-  </si>
-  <si>
-    <t>36</t>
   </si>
   <si>
     <t>CAPEX_ELIGIBLE_ALIGNED_ACTIVITIES</t>
@@ -968,27 +845,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:P58"/>
-  <sheetFormatPr defaultColWidth="255.54296875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="96.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.26953125" customWidth="1"/>
-    <col min="7" max="7" width="32.7265625" customWidth="1"/>
-    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="31.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="28.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="96.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="32.7109375" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1038,7 +915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -1064,8 +941,10 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
@@ -1085,9 +964,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
@@ -1108,9 +987,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
@@ -1131,9 +1010,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
@@ -1154,9 +1033,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -1174,9 +1053,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -1200,9 +1079,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
@@ -1223,9 +1102,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
@@ -1246,9 +1125,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
@@ -1269,9 +1148,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -1292,9 +1171,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -1309,9 +1188,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
         <v>65</v>
@@ -1332,9 +1211,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>164</v>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>65</v>
@@ -1364,9 +1243,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>160</v>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>65</v>
@@ -1396,9 +1275,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>165</v>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>65</v>
@@ -1428,9 +1307,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>166</v>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
+        <v>16</v>
       </c>
       <c r="B18" t="s">
         <v>65</v>
@@ -1457,9 +1336,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>167</v>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" s="2">
+        <v>17</v>
       </c>
       <c r="B19" t="s">
         <v>65</v>
@@ -1486,9 +1365,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>168</v>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20" s="2">
+        <v>18</v>
       </c>
       <c r="B20" t="s">
         <v>65</v>
@@ -1515,9 +1394,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>169</v>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>19</v>
       </c>
       <c r="B21" t="s">
         <v>65</v>
@@ -1544,9 +1423,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>170</v>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>65</v>
@@ -1573,9 +1452,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>171</v>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A23" s="2">
+        <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>65</v>
@@ -1602,9 +1481,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>172</v>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>65</v>
@@ -1631,9 +1510,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>173</v>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>23</v>
       </c>
       <c r="B25" t="s">
         <v>65</v>
@@ -1660,9 +1539,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>174</v>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A26" s="2">
+        <v>24</v>
       </c>
       <c r="B26" t="s">
         <v>65</v>
@@ -1692,27 +1571,27 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>199</v>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A27" s="2">
+        <v>25</v>
       </c>
       <c r="B27" t="s">
         <v>65</v>
       </c>
       <c r="C27" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="D27" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="E27" t="s">
-        <v>208</v>
+        <v>167</v>
       </c>
       <c r="F27" t="s">
-        <v>201</v>
+        <v>161</v>
       </c>
       <c r="G27" t="s">
-        <v>202</v>
+        <v>162</v>
       </c>
       <c r="J27" t="s">
         <v>22</v>
@@ -1724,9 +1603,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>161</v>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A28" s="2">
+        <v>26</v>
       </c>
       <c r="B28" t="s">
         <v>106</v>
@@ -1753,9 +1632,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>162</v>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A29" s="2">
+        <v>27</v>
       </c>
       <c r="B29" t="s">
         <v>106</v>
@@ -1785,9 +1664,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
-        <v>185</v>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A30" s="2">
+        <v>28</v>
       </c>
       <c r="B30" t="s">
         <v>106</v>
@@ -1817,9 +1696,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
-        <v>186</v>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>29</v>
       </c>
       <c r="B31" t="s">
         <v>106</v>
@@ -1849,9 +1728,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>163</v>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A32" s="2">
+        <v>30</v>
       </c>
       <c r="B32" t="s">
         <v>106</v>
@@ -1878,9 +1757,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>176</v>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>31</v>
       </c>
       <c r="B33" t="s">
         <v>106</v>
@@ -1907,9 +1786,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>177</v>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>32</v>
       </c>
       <c r="B34" t="s">
         <v>106</v>
@@ -1936,9 +1815,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
-        <v>178</v>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>33</v>
       </c>
       <c r="B35" t="s">
         <v>106</v>
@@ -1965,9 +1844,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>179</v>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>34</v>
       </c>
       <c r="B36" t="s">
         <v>106</v>
@@ -1994,9 +1873,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
-        <v>180</v>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>35</v>
       </c>
       <c r="B37" t="s">
         <v>106</v>
@@ -2023,9 +1902,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>181</v>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" s="2">
+        <v>36</v>
       </c>
       <c r="B38" t="s">
         <v>106</v>
@@ -2052,9 +1931,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>182</v>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A39" s="2">
+        <v>37</v>
       </c>
       <c r="B39" t="s">
         <v>106</v>
@@ -2081,9 +1960,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>183</v>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>38</v>
       </c>
       <c r="B40" t="s">
         <v>106</v>
@@ -2113,27 +1992,27 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>203</v>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>39</v>
       </c>
       <c r="B41" t="s">
         <v>106</v>
       </c>
       <c r="C41" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="D41" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="E41" t="s">
-        <v>204</v>
+        <v>163</v>
       </c>
       <c r="F41" t="s">
-        <v>205</v>
+        <v>164</v>
       </c>
       <c r="G41" t="s">
-        <v>202</v>
+        <v>162</v>
       </c>
       <c r="J41" t="s">
         <v>22</v>
@@ -2145,9 +2024,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>184</v>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A42" s="2">
+        <v>40</v>
       </c>
       <c r="B42" t="s">
         <v>133</v>
@@ -2174,9 +2053,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
-        <v>187</v>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>133</v>
@@ -2206,9 +2085,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
-        <v>188</v>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A44" s="2">
+        <v>42</v>
       </c>
       <c r="B44" t="s">
         <v>133</v>
@@ -2238,9 +2117,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
-        <v>189</v>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" s="2">
+        <v>43</v>
       </c>
       <c r="B45" t="s">
         <v>133</v>
@@ -2270,9 +2149,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>175</v>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A46" s="2">
+        <v>44</v>
       </c>
       <c r="B46" t="s">
         <v>133</v>
@@ -2299,9 +2178,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>190</v>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>45</v>
       </c>
       <c r="B47" t="s">
         <v>133</v>
@@ -2328,9 +2207,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
-        <v>191</v>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
+        <v>46</v>
       </c>
       <c r="B48" t="s">
         <v>133</v>
@@ -2357,9 +2236,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
-        <v>192</v>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>47</v>
       </c>
       <c r="B49" t="s">
         <v>133</v>
@@ -2386,9 +2265,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
-        <v>193</v>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
+        <v>48</v>
       </c>
       <c r="B50" t="s">
         <v>133</v>
@@ -2415,9 +2294,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
-        <v>194</v>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" s="2">
+        <v>49</v>
       </c>
       <c r="B51" t="s">
         <v>133</v>
@@ -2444,9 +2323,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
-        <v>195</v>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" s="2">
+        <v>50</v>
       </c>
       <c r="B52" t="s">
         <v>133</v>
@@ -2473,9 +2352,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
-        <v>196</v>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A53" s="2">
+        <v>51</v>
       </c>
       <c r="B53" t="s">
         <v>133</v>
@@ -2502,9 +2381,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A54" s="2" t="s">
-        <v>197</v>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A54" s="2">
+        <v>52</v>
       </c>
       <c r="B54" t="s">
         <v>133</v>
@@ -2534,27 +2413,27 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
-        <v>198</v>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A55" s="2">
+        <v>53</v>
       </c>
       <c r="B55" t="s">
         <v>133</v>
       </c>
       <c r="C55" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="D55" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="E55" t="s">
-        <v>206</v>
+        <v>165</v>
       </c>
       <c r="F55" t="s">
-        <v>207</v>
+        <v>166</v>
       </c>
       <c r="G55" t="s">
-        <v>202</v>
+        <v>162</v>
       </c>
       <c r="J55" t="s">
         <v>22</v>
@@ -2566,13 +2445,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
     </row>
   </sheetData>
@@ -2584,30 +2463,55 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
-      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
-      <Description>JFHTZT72FDVU-254938863-279</Description>
-    </_dlc_DocIdUrl>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
-    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100135AEE51B13C7A4784C7A6FB658DD0E0" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c2ccf66da846160ccad12796df698db1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fa7e5010-1311-4096-a344-326d1919664c" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns4="255ceb00-0504-4451-971c-89cf8ee3ad27" xmlns:ns5="953edb04-63dd-49ba-ad7b-e9d17e0e7f06" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd9e9067e801230649229059a2f6238c" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="fa7e5010-1311-4096-a344-326d1919664c"/>
@@ -2853,84 +2757,40 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
+      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
+      <Description>JFHTZT72FDVU-254938863-279</Description>
+    </_dlc_DocIdUrl>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
+    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6E80A2-72F6-4920-8A44-B99818E21D00}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2951,10 +2811,29 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Reordered KPIs in framework input Excel
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93795\Desktop\dataland\dataland\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93814\IdeaProjects\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B95AF64-5C72-42D3-85B6-557E17CEFDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0D564D-7A4E-40C4-B14B-F3C63E38EC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26550" yWindow="1425" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18465" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -845,27 +845,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:P58"/>
-  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="255.59765625" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="96.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="32.7109375" customWidth="1"/>
-    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="96.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.265625" customWidth="1"/>
+    <col min="7" max="7" width="32.73046875" customWidth="1"/>
+    <col min="8" max="8" width="52.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="31.3984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -915,7 +915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -941,7 +941,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -964,7 +964,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -987,7 +987,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1102,7 +1102,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1243,9 +1243,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>65</v>
@@ -1254,16 +1254,16 @@
         <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J16" t="s">
         <v>22</v>
@@ -1275,9 +1275,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
         <v>65</v>
@@ -1286,16 +1286,16 @@
         <v>73</v>
       </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J17" t="s">
         <v>22</v>
@@ -1307,7 +1307,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -1539,7 +1539,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -1664,9 +1664,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A30" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
         <v>106</v>
@@ -1675,16 +1675,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F30" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G30" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J30" t="s">
         <v>22</v>
@@ -1696,9 +1696,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A31" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" t="s">
         <v>106</v>
@@ -1707,16 +1707,16 @@
         <v>73</v>
       </c>
       <c r="D31" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E31" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F31" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J31" t="s">
         <v>22</v>
@@ -1728,7 +1728,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -2085,9 +2085,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A44" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
         <v>133</v>
@@ -2096,16 +2096,16 @@
         <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F44" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G44" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J44" t="s">
         <v>22</v>
@@ -2117,9 +2117,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A45" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B45" t="s">
         <v>133</v>
@@ -2128,16 +2128,16 @@
         <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E45" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F45" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G45" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J45" t="s">
         <v>22</v>
@@ -2149,7 +2149,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -2323,7 +2323,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -2445,13 +2445,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A58" s="2"/>
     </row>
   </sheetData>
@@ -2463,55 +2463,30 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
+      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
+      <Description>JFHTZT72FDVU-254938863-279</Description>
+    </_dlc_DocIdUrl>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
+    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100135AEE51B13C7A4784C7A6FB658DD0E0" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c2ccf66da846160ccad12796df698db1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fa7e5010-1311-4096-a344-326d1919664c" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns4="255ceb00-0504-4451-971c-89cf8ee3ad27" xmlns:ns5="953edb04-63dd-49ba-ad7b-e9d17e0e7f06" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd9e9067e801230649229059a2f6238c" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="fa7e5010-1311-4096-a344-326d1919664c"/>
@@ -2757,40 +2732,84 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
-      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
-      <Description>JFHTZT72FDVU-254938863-279</Description>
-    </_dlc_DocIdUrl>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
-    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6E80A2-72F6-4920-8A44-B99818E21D00}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2811,29 +2830,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Removed subcategory "Eligible or Aligned Activities" from framework input Excel
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93814\IdeaProjects\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0D564D-7A4E-40C4-B14B-F3C63E38EC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D593A41-9867-48A9-A1FE-4928D8C579D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18465" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Framework Data Model'!$A$1:$P$55</definedName>
+  </definedNames>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="168">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -1578,9 +1581,6 @@
       <c r="B27" t="s">
         <v>65</v>
       </c>
-      <c r="C27" t="s">
-        <v>160</v>
-      </c>
       <c r="D27" t="s">
         <v>160</v>
       </c>
@@ -1999,9 +1999,6 @@
       <c r="B41" t="s">
         <v>106</v>
       </c>
-      <c r="C41" t="s">
-        <v>160</v>
-      </c>
       <c r="D41" t="s">
         <v>160</v>
       </c>
@@ -2419,9 +2416,6 @@
       </c>
       <c r="B55" t="s">
         <v>133</v>
-      </c>
-      <c r="C55" t="s">
-        <v>160</v>
       </c>
       <c r="D55" t="s">
         <v>160</v>
@@ -2463,30 +2457,55 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
-      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
-      <Description>JFHTZT72FDVU-254938863-279</Description>
-    </_dlc_DocIdUrl>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
-    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100135AEE51B13C7A4784C7A6FB658DD0E0" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c2ccf66da846160ccad12796df698db1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fa7e5010-1311-4096-a344-326d1919664c" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns4="255ceb00-0504-4451-971c-89cf8ee3ad27" xmlns:ns5="953edb04-63dd-49ba-ad7b-e9d17e0e7f06" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cd9e9067e801230649229059a2f6238c" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="fa7e5010-1311-4096-a344-326d1919664c"/>
@@ -2732,84 +2751,40 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="fa7e5010-1311-4096-a344-326d1919664c">JFHTZT72FDVU-254938863-279</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="fa7e5010-1311-4096-a344-326d1919664c">
+      <Url>https://intranet.d-fine.de/intern/miscellaneous/TemplateFramework/_layouts/15/DocIdRedir.aspx?ID=JFHTZT72FDVU-254938863-279</Url>
+      <Description>JFHTZT72FDVU-254938863-279</Description>
+    </_dlc_DocIdUrl>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Tools xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <Comments xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27" xsi:nil="true"/>
+    <Document_x0020_Category xmlns="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=15.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6E80A2-72F6-4920-8A44-B99818E21D00}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2830,10 +2805,29 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7017BB2C-A3F1-4167-848C-B358A8DC1CB9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="fa7e5010-1311-4096-a344-326d1919664c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="255ceb00-0504-4451-971c-89cf8ee3ad27"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="953edb04-63dd-49ba-ad7b-e9d17e0e7f06"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27E0ED53-E837-41F7-A9C9-5E67E49390EA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0B7321-043A-43C5-BAA4-E29877D5579D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Dala 7164 Fixes for EU Taxo NF 2026 (#1911)
Co-authored-by: Florin Boenkost <276548919+Florin-Boenkost@users.noreply.github.com>
Co-authored-by: Florian Hoeft <245823423+florian-hoeft@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93795\Desktop\dataland\dataland\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93814\IdeaProjects\Dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B95AF64-5C72-42D3-85B6-557E17CEFDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D593A41-9867-48A9-A1FE-4928D8C579D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26550" yWindow="1425" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18465" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Framework Data Model'!$A$1:$P$55</definedName>
+  </definedNames>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="168">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -845,27 +848,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:P58"/>
-  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="255.59765625" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="96.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="32.7109375" customWidth="1"/>
-    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="96.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.265625" customWidth="1"/>
+    <col min="7" max="7" width="32.73046875" customWidth="1"/>
+    <col min="8" max="8" width="52.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="31.3984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -915,7 +918,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -941,7 +944,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -964,7 +967,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -987,7 +990,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1010,7 +1013,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -1033,7 +1036,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1053,7 +1056,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1079,7 +1082,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1102,7 +1105,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1125,7 +1128,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1148,7 +1151,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -1171,7 +1174,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1188,7 +1191,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -1211,7 +1214,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1243,9 +1246,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>65</v>
@@ -1254,16 +1257,16 @@
         <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J16" t="s">
         <v>22</v>
@@ -1275,9 +1278,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
         <v>65</v>
@@ -1286,16 +1289,16 @@
         <v>73</v>
       </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J17" t="s">
         <v>22</v>
@@ -1307,7 +1310,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -1336,7 +1339,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1365,7 +1368,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -1394,7 +1397,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -1423,7 +1426,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -1452,7 +1455,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -1481,7 +1484,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -1510,7 +1513,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -1539,7 +1542,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -1571,16 +1574,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A27" s="2">
         <v>25</v>
       </c>
       <c r="B27" t="s">
         <v>65</v>
       </c>
-      <c r="C27" t="s">
-        <v>160</v>
-      </c>
       <c r="D27" t="s">
         <v>160</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -1664,9 +1664,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A30" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
         <v>106</v>
@@ -1675,16 +1675,16 @@
         <v>73</v>
       </c>
       <c r="D30" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F30" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G30" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J30" t="s">
         <v>22</v>
@@ -1696,9 +1696,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A31" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" t="s">
         <v>106</v>
@@ -1707,16 +1707,16 @@
         <v>73</v>
       </c>
       <c r="D31" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E31" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F31" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J31" t="s">
         <v>22</v>
@@ -1728,7 +1728,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -1992,16 +1992,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A41" s="2">
         <v>39</v>
       </c>
       <c r="B41" t="s">
         <v>106</v>
       </c>
-      <c r="C41" t="s">
-        <v>160</v>
-      </c>
       <c r="D41" t="s">
         <v>160</v>
       </c>
@@ -2024,7 +2021,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -2053,7 +2050,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -2085,9 +2082,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A44" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
         <v>133</v>
@@ -2096,16 +2093,16 @@
         <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F44" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G44" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J44" t="s">
         <v>22</v>
@@ -2117,9 +2114,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A45" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B45" t="s">
         <v>133</v>
@@ -2128,16 +2125,16 @@
         <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E45" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F45" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G45" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J45" t="s">
         <v>22</v>
@@ -2149,7 +2146,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -2178,7 +2175,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -2207,7 +2204,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -2236,7 +2233,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -2265,7 +2262,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -2294,7 +2291,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -2323,7 +2320,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -2352,7 +2349,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -2381,7 +2378,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -2413,16 +2410,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A55" s="2">
         <v>53</v>
       </c>
       <c r="B55" t="s">
         <v>133</v>
       </c>
-      <c r="C55" t="s">
-        <v>160</v>
-      </c>
       <c r="D55" t="s">
         <v>160</v>
       </c>
@@ -2445,13 +2439,13 @@
         <v>45</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A58" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added calculation rules to Excel and ran framework-toolbox
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E16E7C-B9EF-48C6-94AF-ADDAFFDB7D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374B4AA-9680-4CEC-B0FA-23313FE1F6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="173">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -533,13 +533,22 @@
   <si>
     <t>Existence of due diligence processes to identify, prevent, mitigate and address adverse human rights impacts.
 Linked to Regulation (EU) 2022/1288, Annex I, Table 3, Adverse impact on sustainability factor 10</t>
+  </si>
+  <si>
+    <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentRevenueNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentRevenueAlignedActivities]</t>
+  </si>
+  <si>
+    <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentCapexNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentCapexAlignedActivities]</t>
+  </si>
+  <si>
+    <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentOpexNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentOpexAlignedActivities]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -550,6 +559,11 @@
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF172B4D"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -594,7 +608,7 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -607,6 +621,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -854,7 +871,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Q58"/>
-  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -875,7 +892,7 @@
     <col min="17" max="17" width="28.5703125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -928,7 +945,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -954,7 +971,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -977,7 +994,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -1000,7 +1017,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1026,7 +1043,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -1049,7 +1066,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1069,7 +1086,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1095,7 +1112,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="38.25">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1118,7 +1135,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1141,7 +1158,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1164,7 +1181,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="51">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -1187,7 +1204,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1204,7 +1221,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -1227,7 +1244,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1259,7 +1276,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1291,7 +1308,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17">
       <c r="A17" s="2">
         <v>14</v>
       </c>
@@ -1323,7 +1340,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -1352,7 +1369,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1381,7 +1398,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -1410,7 +1427,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -1439,7 +1456,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -1468,7 +1485,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -1497,7 +1514,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -1526,7 +1543,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -1555,7 +1572,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -1587,7 +1604,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -1615,8 +1632,11 @@
       <c r="O27" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="Q27" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -1645,7 +1665,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -1677,7 +1697,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1709,7 +1729,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17">
       <c r="A31" s="2">
         <v>28</v>
       </c>
@@ -1741,7 +1761,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -1770,7 +1790,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -1799,7 +1819,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -1828,7 +1848,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -1857,7 +1877,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -1886,7 +1906,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -1915,7 +1935,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -1944,7 +1964,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -1973,7 +1993,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -2005,7 +2025,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -2033,8 +2053,11 @@
       <c r="O41" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="Q41" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -2063,7 +2086,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -2095,7 +2118,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2127,7 +2150,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17">
       <c r="A45" s="2">
         <v>42</v>
       </c>
@@ -2159,7 +2182,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -2188,7 +2211,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -2217,7 +2240,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -2246,7 +2269,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -2275,7 +2298,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -2304,7 +2327,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -2333,7 +2356,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -2362,7 +2385,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -2391,7 +2414,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -2423,7 +2446,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -2451,14 +2474,17 @@
       <c r="O55" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="Q55" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17">
       <c r="A58" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed template diagnostic warning when option column is used
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374B4AA-9680-4CEC-B0FA-23313FE1F6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FDA3FB-61F3-4EF5-AA26-6C182AB47FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="196">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -542,6 +542,75 @@
   </si>
   <si>
     <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentOpexNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentOpexAlignedActivities]</t>
+  </si>
+  <si>
+    <t>Relative Share of Nuclear Activities in Percent - Eligible</t>
+  </si>
+  <si>
+    <t>Relative Share of Nuclear Activities in Percent - Aligned</t>
+  </si>
+  <si>
+    <t>Relative Share of Fossil Gas Activities in Percent - Eligible</t>
+  </si>
+  <si>
+    <t>Relative Share of Fossil Gas Activities in Percent - Aligned</t>
+  </si>
+  <si>
+    <t>REV_NUCLEAR_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>REV_NUCLEAR_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>REV_GAS_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>REV_GAS_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-eligible nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-aligned nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-eligible fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-aligned fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>NoUpload</t>
+  </si>
+  <si>
+    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentRevenueEligibleOrAlignedActivities], EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentRevenueAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentRevenueNonAlignedActivities]</t>
+  </si>
+  <si>
+    <t>CAPEX_NUCLEAR_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-eligible nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>CAPEX_NUCLEAR_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-aligned nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>CAPEX_GAS_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-eligible fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>CAPEX_GAS_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-aligned fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentCapexEligibleOrAlignedActivities], EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentCapexAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentCapexNonAlignedActivities]</t>
   </si>
 </sst>
 </file>
@@ -870,7 +939,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Q58"/>
+  <dimension ref="A1:Q66"/>
   <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -1573,27 +1642,25 @@
       </c>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="2">
-        <v>24</v>
-      </c>
+      <c r="A26" s="2"/>
       <c r="B26" t="s">
         <v>61</v>
       </c>
-      <c r="C26" t="s">
-        <v>102</v>
-      </c>
       <c r="D26" t="s">
-        <v>67</v>
+        <v>173</v>
       </c>
       <c r="E26" t="s">
-        <v>103</v>
+        <v>177</v>
       </c>
       <c r="F26" t="s">
-        <v>104</v>
+        <v>181</v>
       </c>
       <c r="G26" t="s">
         <v>70</v>
       </c>
+      <c r="H26" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="J26" t="s">
         <v>23</v>
       </c>
@@ -1603,25 +1670,29 @@
       <c r="O26" t="s">
         <v>71</v>
       </c>
+      <c r="Q26" s="3" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="27" spans="1:17">
-      <c r="A27" s="2">
-        <v>25</v>
-      </c>
+      <c r="A27" s="2"/>
       <c r="B27" t="s">
         <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>174</v>
       </c>
       <c r="E27" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="F27" t="s">
-        <v>107</v>
+        <v>182</v>
       </c>
       <c r="G27" t="s">
-        <v>108</v>
+        <v>70</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J27" t="s">
         <v>23</v>
@@ -1633,27 +1704,28 @@
         <v>71</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
     </row>
     <row r="28" spans="1:17">
-      <c r="A28" s="2">
-        <v>26</v>
-      </c>
+      <c r="A28" s="2"/>
       <c r="B28" t="s">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>62</v>
+        <v>175</v>
       </c>
       <c r="E28" t="s">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="F28" t="s">
-        <v>111</v>
+        <v>183</v>
       </c>
       <c r="G28" t="s">
-        <v>65</v>
+        <v>70</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J28" t="s">
         <v>23</v>
@@ -1664,29 +1736,30 @@
       <c r="O28" t="s">
         <v>71</v>
       </c>
+      <c r="Q28" s="3" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="29" spans="1:17">
-      <c r="A29" s="2">
-        <v>27</v>
-      </c>
+      <c r="A29" s="2"/>
       <c r="B29" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>67</v>
+        <v>176</v>
       </c>
       <c r="E29" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="F29" t="s">
-        <v>113</v>
+        <v>184</v>
       </c>
       <c r="G29" t="s">
         <v>70</v>
       </c>
+      <c r="H29" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="J29" t="s">
         <v>23</v>
       </c>
@@ -1695,29 +1768,32 @@
       </c>
       <c r="O29" t="s">
         <v>71</v>
+      </c>
+      <c r="Q29" s="3" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" s="2">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="D30" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E30" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="F30" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G30" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J30" t="s">
         <v>23</v>
@@ -1731,25 +1807,22 @@
     </row>
     <row r="31" spans="1:17">
       <c r="A31" s="2">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>109</v>
-      </c>
-      <c r="C31" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="E31" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="F31" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="G31" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="J31" t="s">
         <v>23</v>
@@ -1759,26 +1832,29 @@
       </c>
       <c r="O31" t="s">
         <v>71</v>
+      </c>
+      <c r="Q31" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:17">
       <c r="A32" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B32" t="s">
         <v>109</v>
       </c>
       <c r="D32" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E32" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="G32" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J32" t="s">
         <v>23</v>
@@ -1792,19 +1868,22 @@
     </row>
     <row r="33" spans="1:17">
       <c r="A33" s="2">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B33" t="s">
         <v>109</v>
       </c>
+      <c r="C33" t="s">
+        <v>66</v>
+      </c>
       <c r="D33" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="E33" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="F33" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="G33" t="s">
         <v>70</v>
@@ -1821,22 +1900,25 @@
     </row>
     <row r="34" spans="1:17">
       <c r="A34" s="2">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B34" t="s">
         <v>109</v>
       </c>
+      <c r="C34" t="s">
+        <v>72</v>
+      </c>
       <c r="D34" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="E34" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="G34" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J34" t="s">
         <v>23</v>
@@ -1850,19 +1932,22 @@
     </row>
     <row r="35" spans="1:17">
       <c r="A35" s="2">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B35" t="s">
         <v>109</v>
       </c>
+      <c r="C35" t="s">
+        <v>72</v>
+      </c>
       <c r="D35" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="E35" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="F35" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="G35" t="s">
         <v>70</v>
@@ -1879,19 +1964,19 @@
     </row>
     <row r="36" spans="1:17">
       <c r="A36" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B36" t="s">
         <v>109</v>
       </c>
       <c r="D36" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E36" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="F36" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="G36" t="s">
         <v>70</v>
@@ -1908,19 +1993,19 @@
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="2">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B37" t="s">
         <v>109</v>
       </c>
       <c r="D37" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E37" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F37" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="G37" t="s">
         <v>70</v>
@@ -1937,19 +2022,19 @@
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="2">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B38" t="s">
         <v>109</v>
       </c>
       <c r="D38" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="E38" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="F38" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="G38" t="s">
         <v>70</v>
@@ -1966,19 +2051,19 @@
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="2">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B39" t="s">
         <v>109</v>
       </c>
       <c r="D39" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="E39" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="F39" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="G39" t="s">
         <v>70</v>
@@ -1995,22 +2080,19 @@
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
         <v>109</v>
       </c>
-      <c r="C40" t="s">
-        <v>102</v>
-      </c>
       <c r="D40" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="F40" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="G40" t="s">
         <v>70</v>
@@ -2027,22 +2109,22 @@
     </row>
     <row r="41" spans="1:17">
       <c r="A41" s="2">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B41" t="s">
         <v>109</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="E41" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="G41" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="J41" t="s">
         <v>23</v>
@@ -2052,29 +2134,26 @@
       </c>
       <c r="O41" t="s">
         <v>71</v>
-      </c>
-      <c r="Q41" s="3" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="2">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D42" t="s">
-        <v>62</v>
+        <v>96</v>
       </c>
       <c r="E42" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="F42" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="G42" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J42" t="s">
         <v>23</v>
@@ -2088,22 +2167,19 @@
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="2">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B43" t="s">
-        <v>138</v>
-      </c>
-      <c r="C43" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="D43" t="s">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="E43" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="F43" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="G43" t="s">
         <v>70</v>
@@ -2119,26 +2195,24 @@
       </c>
     </row>
     <row r="44" spans="1:17">
-      <c r="A44" s="2">
-        <v>43</v>
-      </c>
+      <c r="A44" s="2"/>
       <c r="B44" t="s">
-        <v>138</v>
-      </c>
-      <c r="C44" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="D44" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="E44" t="s">
-        <v>143</v>
+        <v>187</v>
       </c>
       <c r="F44" t="s">
-        <v>144</v>
-      </c>
-      <c r="G44" t="s">
-        <v>65</v>
+        <v>188</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J44" t="s">
         <v>23</v>
@@ -2149,28 +2223,29 @@
       <c r="O44" t="s">
         <v>71</v>
       </c>
+      <c r="Q44" s="3" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="45" spans="1:17">
-      <c r="A45" s="2">
-        <v>42</v>
-      </c>
+      <c r="A45" s="2"/>
       <c r="B45" t="s">
-        <v>138</v>
-      </c>
-      <c r="C45" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="D45" t="s">
-        <v>67</v>
+        <v>174</v>
       </c>
       <c r="E45" t="s">
-        <v>145</v>
+        <v>189</v>
       </c>
       <c r="F45" t="s">
-        <v>146</v>
-      </c>
-      <c r="G45" t="s">
-        <v>70</v>
+        <v>190</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J45" t="s">
         <v>23</v>
@@ -2181,25 +2256,29 @@
       <c r="O45" t="s">
         <v>71</v>
       </c>
+      <c r="Q45" s="3" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" s="2">
-        <v>44</v>
-      </c>
+      <c r="A46" s="2"/>
       <c r="B46" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D46" t="s">
-        <v>78</v>
+        <v>175</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>191</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
-      </c>
-      <c r="G46" t="s">
-        <v>70</v>
+        <v>192</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J46" t="s">
         <v>23</v>
@@ -2210,25 +2289,29 @@
       <c r="O46" t="s">
         <v>71</v>
       </c>
+      <c r="Q46" s="3" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="47" spans="1:17">
-      <c r="A47" s="2">
-        <v>45</v>
-      </c>
+      <c r="A47" s="2"/>
       <c r="B47" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D47" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
       <c r="E47" t="s">
-        <v>149</v>
+        <v>193</v>
       </c>
       <c r="F47" t="s">
-        <v>150</v>
-      </c>
-      <c r="G47" t="s">
-        <v>70</v>
+        <v>194</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J47" t="s">
         <v>23</v>
@@ -2238,23 +2321,29 @@
       </c>
       <c r="O47" t="s">
         <v>71</v>
+      </c>
+      <c r="Q47" s="3" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:17">
       <c r="A48" s="2">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B48" t="s">
-        <v>138</v>
+        <v>109</v>
+      </c>
+      <c r="C48" t="s">
+        <v>102</v>
       </c>
       <c r="D48" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="E48" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="F48" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="G48" t="s">
         <v>70</v>
@@ -2271,22 +2360,22 @@
     </row>
     <row r="49" spans="1:17">
       <c r="A49" s="2">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B49" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D49" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E49" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="F49" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="G49" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="J49" t="s">
         <v>23</v>
@@ -2296,26 +2385,29 @@
       </c>
       <c r="O49" t="s">
         <v>71</v>
+      </c>
+      <c r="Q49" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="2">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B50" t="s">
         <v>138</v>
       </c>
       <c r="D50" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E50" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="F50" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="G50" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J50" t="s">
         <v>23</v>
@@ -2329,19 +2421,22 @@
     </row>
     <row r="51" spans="1:17">
       <c r="A51" s="2">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B51" t="s">
         <v>138</v>
       </c>
+      <c r="C51" t="s">
+        <v>66</v>
+      </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="E51" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="F51" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="G51" t="s">
         <v>70</v>
@@ -2358,22 +2453,25 @@
     </row>
     <row r="52" spans="1:17">
       <c r="A52" s="2">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B52" t="s">
         <v>138</v>
       </c>
+      <c r="C52" t="s">
+        <v>72</v>
+      </c>
       <c r="D52" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E52" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="F52" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="G52" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J52" t="s">
         <v>23</v>
@@ -2387,19 +2485,22 @@
     </row>
     <row r="53" spans="1:17">
       <c r="A53" s="2">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B53" t="s">
         <v>138</v>
       </c>
+      <c r="C53" t="s">
+        <v>72</v>
+      </c>
       <c r="D53" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="E53" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="F53" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="G53" t="s">
         <v>70</v>
@@ -2416,22 +2517,19 @@
     </row>
     <row r="54" spans="1:17">
       <c r="A54" s="2">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="B54" t="s">
         <v>138</v>
       </c>
-      <c r="C54" t="s">
-        <v>102</v>
-      </c>
       <c r="D54" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E54" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="F54" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="G54" t="s">
         <v>70</v>
@@ -2448,44 +2546,279 @@
     </row>
     <row r="55" spans="1:17">
       <c r="A55" s="2">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B55" t="s">
         <v>138</v>
       </c>
       <c r="D55" t="s">
+        <v>81</v>
+      </c>
+      <c r="E55" t="s">
+        <v>149</v>
+      </c>
+      <c r="F55" t="s">
+        <v>150</v>
+      </c>
+      <c r="G55" t="s">
+        <v>70</v>
+      </c>
+      <c r="J55" t="s">
+        <v>23</v>
+      </c>
+      <c r="N55" t="s">
+        <v>71</v>
+      </c>
+      <c r="O55" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
+      <c r="A56" s="2">
+        <v>46</v>
+      </c>
+      <c r="B56" t="s">
+        <v>138</v>
+      </c>
+      <c r="D56" t="s">
+        <v>84</v>
+      </c>
+      <c r="E56" t="s">
+        <v>151</v>
+      </c>
+      <c r="F56" t="s">
+        <v>152</v>
+      </c>
+      <c r="G56" t="s">
+        <v>70</v>
+      </c>
+      <c r="J56" t="s">
+        <v>23</v>
+      </c>
+      <c r="N56" t="s">
+        <v>71</v>
+      </c>
+      <c r="O56" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17">
+      <c r="A57" s="2">
+        <v>47</v>
+      </c>
+      <c r="B57" t="s">
+        <v>138</v>
+      </c>
+      <c r="D57" t="s">
+        <v>87</v>
+      </c>
+      <c r="E57" t="s">
+        <v>153</v>
+      </c>
+      <c r="F57" t="s">
+        <v>154</v>
+      </c>
+      <c r="G57" t="s">
+        <v>70</v>
+      </c>
+      <c r="J57" t="s">
+        <v>23</v>
+      </c>
+      <c r="N57" t="s">
+        <v>71</v>
+      </c>
+      <c r="O57" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17">
+      <c r="A58" s="2">
+        <v>48</v>
+      </c>
+      <c r="B58" t="s">
+        <v>138</v>
+      </c>
+      <c r="D58" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" t="s">
+        <v>155</v>
+      </c>
+      <c r="F58" t="s">
+        <v>156</v>
+      </c>
+      <c r="G58" t="s">
+        <v>70</v>
+      </c>
+      <c r="J58" t="s">
+        <v>23</v>
+      </c>
+      <c r="N58" t="s">
+        <v>71</v>
+      </c>
+      <c r="O58" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17">
+      <c r="A59" s="2">
+        <v>49</v>
+      </c>
+      <c r="B59" t="s">
+        <v>138</v>
+      </c>
+      <c r="D59" t="s">
+        <v>93</v>
+      </c>
+      <c r="E59" t="s">
+        <v>157</v>
+      </c>
+      <c r="F59" t="s">
+        <v>158</v>
+      </c>
+      <c r="G59" t="s">
+        <v>70</v>
+      </c>
+      <c r="J59" t="s">
+        <v>23</v>
+      </c>
+      <c r="N59" t="s">
+        <v>71</v>
+      </c>
+      <c r="O59" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17">
+      <c r="A60" s="2">
+        <v>50</v>
+      </c>
+      <c r="B60" t="s">
+        <v>138</v>
+      </c>
+      <c r="D60" t="s">
+        <v>96</v>
+      </c>
+      <c r="E60" t="s">
+        <v>159</v>
+      </c>
+      <c r="F60" t="s">
+        <v>160</v>
+      </c>
+      <c r="G60" t="s">
+        <v>70</v>
+      </c>
+      <c r="J60" t="s">
+        <v>23</v>
+      </c>
+      <c r="N60" t="s">
+        <v>71</v>
+      </c>
+      <c r="O60" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17">
+      <c r="A61" s="2">
+        <v>51</v>
+      </c>
+      <c r="B61" t="s">
+        <v>138</v>
+      </c>
+      <c r="D61" t="s">
+        <v>99</v>
+      </c>
+      <c r="E61" t="s">
+        <v>161</v>
+      </c>
+      <c r="F61" t="s">
+        <v>162</v>
+      </c>
+      <c r="G61" t="s">
+        <v>70</v>
+      </c>
+      <c r="J61" t="s">
+        <v>23</v>
+      </c>
+      <c r="N61" t="s">
+        <v>71</v>
+      </c>
+      <c r="O61" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17">
+      <c r="A62" s="2">
+        <v>52</v>
+      </c>
+      <c r="B62" t="s">
+        <v>138</v>
+      </c>
+      <c r="C62" t="s">
+        <v>102</v>
+      </c>
+      <c r="D62" t="s">
+        <v>67</v>
+      </c>
+      <c r="E62" t="s">
+        <v>163</v>
+      </c>
+      <c r="F62" t="s">
+        <v>164</v>
+      </c>
+      <c r="G62" t="s">
+        <v>70</v>
+      </c>
+      <c r="J62" t="s">
+        <v>23</v>
+      </c>
+      <c r="N62" t="s">
+        <v>71</v>
+      </c>
+      <c r="O62" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17">
+      <c r="A63" s="2">
+        <v>53</v>
+      </c>
+      <c r="B63" t="s">
+        <v>138</v>
+      </c>
+      <c r="D63" t="s">
         <v>105</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E63" t="s">
         <v>165</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F63" t="s">
         <v>166</v>
       </c>
-      <c r="G55" t="s">
+      <c r="G63" t="s">
         <v>108</v>
       </c>
-      <c r="J55" t="s">
-        <v>23</v>
-      </c>
-      <c r="N55" t="s">
-        <v>71</v>
-      </c>
-      <c r="O55" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q55" s="5" t="s">
+      <c r="J63" t="s">
+        <v>23</v>
+      </c>
+      <c r="N63" t="s">
+        <v>71</v>
+      </c>
+      <c r="O63" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q63" s="5" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="56" spans="1:17">
-      <c r="A56" s="2"/>
-    </row>
-    <row r="57" spans="1:17">
-      <c r="A57" s="2"/>
-    </row>
-    <row r="58" spans="1:17">
-      <c r="A58" s="2"/>
+    <row r="64" spans="1:17">
+      <c r="A64" s="2"/>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="2"/>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adapted framework excel file
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FDA3FB-61F3-4EF5-AA26-6C182AB47FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C62AF0D-6D67-4593-9C94-6EA1A14B3343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -583,9 +583,6 @@
     <t>NoUpload</t>
   </si>
   <si>
-    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentRevenueEligibleOrAlignedActivities], EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentRevenueAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentRevenueNonAlignedActivities]</t>
-  </si>
-  <si>
     <t>CAPEX_NUCLEAR_ELIGIBLE_PCT</t>
   </si>
   <si>
@@ -610,7 +607,10 @@
     <t>Relative share of the CapEx that is associated with taxonomy-aligned fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
   </si>
   <si>
-    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentCapexEligibleOrAlignedActivities], EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentCapexAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentCapexNonAlignedActivities]</t>
+    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentRevenueEligibleOrAlignedActivities]; EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentRevenueAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentRevenueNonAlignedActivities]</t>
+  </si>
+  <si>
+    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentCapexEligibleOrAlignedActivities]; EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentCapexAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentCapexNonAlignedActivities]</t>
   </si>
 </sst>
 </file>
@@ -1347,7 +1347,7 @@
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>61</v>
@@ -1379,7 +1379,7 @@
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>61</v>
@@ -1642,7 +1642,9 @@
       </c>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="2"/>
+      <c r="A26" s="2">
+        <v>24</v>
+      </c>
       <c r="B26" t="s">
         <v>61</v>
       </c>
@@ -1671,11 +1673,13 @@
         <v>71</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" spans="1:17">
-      <c r="A27" s="2"/>
+      <c r="A27" s="2">
+        <v>25</v>
+      </c>
       <c r="B27" t="s">
         <v>61</v>
       </c>
@@ -1704,11 +1708,13 @@
         <v>71</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:17">
-      <c r="A28" s="2"/>
+      <c r="A28" s="2">
+        <v>26</v>
+      </c>
       <c r="B28" t="s">
         <v>61</v>
       </c>
@@ -1737,11 +1743,13 @@
         <v>71</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:17">
-      <c r="A29" s="2"/>
+      <c r="A29" s="2">
+        <v>27</v>
+      </c>
       <c r="B29" t="s">
         <v>61</v>
       </c>
@@ -1770,12 +1778,12 @@
         <v>71</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" s="2">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
         <v>61</v>
@@ -1807,7 +1815,7 @@
     </row>
     <row r="31" spans="1:17">
       <c r="A31" s="2">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B31" t="s">
         <v>61</v>
@@ -1839,7 +1847,7 @@
     </row>
     <row r="32" spans="1:17">
       <c r="A32" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
         <v>109</v>
@@ -1868,7 +1876,7 @@
     </row>
     <row r="33" spans="1:17">
       <c r="A33" s="2">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
         <v>109</v>
@@ -1900,7 +1908,7 @@
     </row>
     <row r="34" spans="1:17">
       <c r="A34" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
         <v>109</v>
@@ -1932,7 +1940,7 @@
     </row>
     <row r="35" spans="1:17">
       <c r="A35" s="2">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B35" t="s">
         <v>109</v>
@@ -1964,7 +1972,7 @@
     </row>
     <row r="36" spans="1:17">
       <c r="A36" s="2">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
         <v>109</v>
@@ -1993,7 +2001,7 @@
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="2">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
         <v>109</v>
@@ -2022,7 +2030,7 @@
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="2">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B38" t="s">
         <v>109</v>
@@ -2051,7 +2059,7 @@
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B39" t="s">
         <v>109</v>
@@ -2080,7 +2088,7 @@
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="2">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B40" t="s">
         <v>109</v>
@@ -2109,7 +2117,7 @@
     </row>
     <row r="41" spans="1:17">
       <c r="A41" s="2">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B41" t="s">
         <v>109</v>
@@ -2138,7 +2146,7 @@
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="2">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B42" t="s">
         <v>109</v>
@@ -2167,7 +2175,7 @@
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>109</v>
@@ -2195,7 +2203,9 @@
       </c>
     </row>
     <row r="44" spans="1:17">
-      <c r="A44" s="2"/>
+      <c r="A44" s="2">
+        <v>42</v>
+      </c>
       <c r="B44" t="s">
         <v>109</v>
       </c>
@@ -2203,10 +2213,10 @@
         <v>173</v>
       </c>
       <c r="E44" t="s">
+        <v>186</v>
+      </c>
+      <c r="F44" t="s">
         <v>187</v>
-      </c>
-      <c r="F44" t="s">
-        <v>188</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>70</v>
@@ -2228,7 +2238,9 @@
       </c>
     </row>
     <row r="45" spans="1:17">
-      <c r="A45" s="2"/>
+      <c r="A45" s="2">
+        <v>43</v>
+      </c>
       <c r="B45" t="s">
         <v>109</v>
       </c>
@@ -2236,10 +2248,10 @@
         <v>174</v>
       </c>
       <c r="E45" t="s">
+        <v>188</v>
+      </c>
+      <c r="F45" t="s">
         <v>189</v>
-      </c>
-      <c r="F45" t="s">
-        <v>190</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>70</v>
@@ -2261,7 +2273,9 @@
       </c>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" s="2"/>
+      <c r="A46" s="2">
+        <v>44</v>
+      </c>
       <c r="B46" t="s">
         <v>109</v>
       </c>
@@ -2269,10 +2283,10 @@
         <v>175</v>
       </c>
       <c r="E46" t="s">
+        <v>190</v>
+      </c>
+      <c r="F46" t="s">
         <v>191</v>
-      </c>
-      <c r="F46" t="s">
-        <v>192</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>70</v>
@@ -2294,7 +2308,9 @@
       </c>
     </row>
     <row r="47" spans="1:17">
-      <c r="A47" s="2"/>
+      <c r="A47" s="2">
+        <v>45</v>
+      </c>
       <c r="B47" t="s">
         <v>109</v>
       </c>
@@ -2302,10 +2318,10 @@
         <v>176</v>
       </c>
       <c r="E47" t="s">
+        <v>192</v>
+      </c>
+      <c r="F47" t="s">
         <v>193</v>
-      </c>
-      <c r="F47" t="s">
-        <v>194</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>70</v>
@@ -2328,7 +2344,7 @@
     </row>
     <row r="48" spans="1:17">
       <c r="A48" s="2">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B48" t="s">
         <v>109</v>
@@ -2360,7 +2376,7 @@
     </row>
     <row r="49" spans="1:17">
       <c r="A49" s="2">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B49" t="s">
         <v>109</v>
@@ -2392,7 +2408,7 @@
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="2">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B50" t="s">
         <v>138</v>
@@ -2421,7 +2437,7 @@
     </row>
     <row r="51" spans="1:17">
       <c r="A51" s="2">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B51" t="s">
         <v>138</v>
@@ -2453,7 +2469,7 @@
     </row>
     <row r="52" spans="1:17">
       <c r="A52" s="2">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B52" t="s">
         <v>138</v>
@@ -2485,7 +2501,7 @@
     </row>
     <row r="53" spans="1:17">
       <c r="A53" s="2">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="B53" t="s">
         <v>138</v>
@@ -2517,7 +2533,7 @@
     </row>
     <row r="54" spans="1:17">
       <c r="A54" s="2">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B54" t="s">
         <v>138</v>
@@ -2546,7 +2562,7 @@
     </row>
     <row r="55" spans="1:17">
       <c r="A55" s="2">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B55" t="s">
         <v>138</v>
@@ -2575,7 +2591,7 @@
     </row>
     <row r="56" spans="1:17">
       <c r="A56" s="2">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
         <v>138</v>
@@ -2604,7 +2620,7 @@
     </row>
     <row r="57" spans="1:17">
       <c r="A57" s="2">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B57" t="s">
         <v>138</v>
@@ -2633,7 +2649,7 @@
     </row>
     <row r="58" spans="1:17">
       <c r="A58" s="2">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B58" t="s">
         <v>138</v>
@@ -2662,7 +2678,7 @@
     </row>
     <row r="59" spans="1:17">
       <c r="A59" s="2">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B59" t="s">
         <v>138</v>
@@ -2691,7 +2707,7 @@
     </row>
     <row r="60" spans="1:17">
       <c r="A60" s="2">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B60" t="s">
         <v>138</v>
@@ -2720,7 +2736,7 @@
     </row>
     <row r="61" spans="1:17">
       <c r="A61" s="2">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B61" t="s">
         <v>138</v>
@@ -2749,7 +2765,7 @@
     </row>
     <row r="62" spans="1:17">
       <c r="A62" s="2">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B62" t="s">
         <v>138</v>
@@ -2781,7 +2797,7 @@
     </row>
     <row r="63" spans="1:17">
       <c r="A63" s="2">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B63" t="s">
         <v>138</v>

</xml_diff>

<commit_message>
DALA-6987: support for calculation creation of 2026 non financials activities (#2012)
---------

Co-authored-by: Dominik Tschimmel <296276725+DominikTschimmel-d-fine@users.noreply.github.com>
Co-authored-by: SiegfriedSobkowiak <71646830+SiegfriedSobkowiak@users.noreply.github.com>
Co-authored-by: StephanWezorke <186339469+StephanWezorke@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E16E7C-B9EF-48C6-94AF-ADDAFFDB7D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374B4AA-9680-4CEC-B0FA-23313FE1F6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="173">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -533,13 +533,22 @@
   <si>
     <t>Existence of due diligence processes to identify, prevent, mitigate and address adverse human rights impacts.
 Linked to Regulation (EU) 2022/1288, Annex I, Table 3, Adverse impact on sustainability factor 10</t>
+  </si>
+  <si>
+    <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentRevenueNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentRevenueAlignedActivities]</t>
+  </si>
+  <si>
+    <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentCapexNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentCapexAlignedActivities]</t>
+  </si>
+  <si>
+    <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentOpexNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentOpexAlignedActivities]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -550,6 +559,11 @@
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF172B4D"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -594,7 +608,7 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -607,6 +621,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -854,7 +871,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Q58"/>
-  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -875,7 +892,7 @@
     <col min="17" max="17" width="28.5703125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -928,7 +945,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -954,7 +971,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -977,7 +994,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -1000,7 +1017,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1026,7 +1043,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -1049,7 +1066,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1069,7 +1086,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1095,7 +1112,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="38.25">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1118,7 +1135,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1141,7 +1158,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1164,7 +1181,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="51">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -1187,7 +1204,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1204,7 +1221,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -1227,7 +1244,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1259,7 +1276,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1291,7 +1308,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17">
       <c r="A17" s="2">
         <v>14</v>
       </c>
@@ -1323,7 +1340,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -1352,7 +1369,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1381,7 +1398,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -1410,7 +1427,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -1439,7 +1456,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -1468,7 +1485,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -1497,7 +1514,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -1526,7 +1543,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -1555,7 +1572,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -1587,7 +1604,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -1615,8 +1632,11 @@
       <c r="O27" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="Q27" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -1645,7 +1665,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -1677,7 +1697,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1709,7 +1729,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17">
       <c r="A31" s="2">
         <v>28</v>
       </c>
@@ -1741,7 +1761,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -1770,7 +1790,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -1799,7 +1819,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -1828,7 +1848,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -1857,7 +1877,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -1886,7 +1906,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -1915,7 +1935,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -1944,7 +1964,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -1973,7 +1993,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -2005,7 +2025,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -2033,8 +2053,11 @@
       <c r="O41" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="Q41" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -2063,7 +2086,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -2095,7 +2118,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2127,7 +2150,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17">
       <c r="A45" s="2">
         <v>42</v>
       </c>
@@ -2159,7 +2182,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -2188,7 +2211,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -2217,7 +2240,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -2246,7 +2269,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -2275,7 +2298,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -2304,7 +2327,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -2333,7 +2356,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -2362,7 +2385,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -2391,7 +2414,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -2423,7 +2446,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -2451,14 +2474,17 @@
       <c r="O55" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="Q55" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17">
       <c r="A58" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dala 7363 nuclear and gas data points for eu taxo non financial 2026 (#2019)
Co-authored-by: Dominik Tschimmel <296276725+DominikTschimmel-d-fine@users.noreply.github.com>
Co-authored-by: SiegfriedSobkowiak <71646830+SiegfriedSobkowiak@users.noreply.github.com>
Co-authored-by: StephanWezorke <186339469+StephanWezorke@users.noreply.github.com>
Co-authored-by: florian-hoeft <245823423+florian-hoeft@users.noreply.github.com>
Co-authored-by: Joshua Köck <49119664+JoshuaKoeck@users.noreply.github.com>
Co-authored-by: Paul Kogler <305446092+PauliKogler@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
+++ b/dataland-framework-toolbox/inputs/eutaxonomy-non-financials-2026-73/eutaxonomy-non-financials-2026-73.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\eutaxonomy-non-financials-2026-73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374B4AA-9680-4CEC-B0FA-23313FE1F6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C62AF0D-6D67-4593-9C94-6EA1A14B3343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="196">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -542,6 +542,75 @@
   </si>
   <si>
     <t>EuTaxonomyActivityMerge: [extendedEuTaxonomyNonAlignedActivitiesComponentOpexNonAlignedActivities, extendedEuTaxonomyAlignedActivitiesComponentOpexAlignedActivities]</t>
+  </si>
+  <si>
+    <t>Relative Share of Nuclear Activities in Percent - Eligible</t>
+  </si>
+  <si>
+    <t>Relative Share of Nuclear Activities in Percent - Aligned</t>
+  </si>
+  <si>
+    <t>Relative Share of Fossil Gas Activities in Percent - Eligible</t>
+  </si>
+  <si>
+    <t>Relative Share of Fossil Gas Activities in Percent - Aligned</t>
+  </si>
+  <si>
+    <t>REV_NUCLEAR_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>REV_NUCLEAR_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>REV_GAS_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>REV_GAS_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-eligible nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-aligned nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-eligible fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>Relative share of the revenue that is associated with taxonomy-aligned fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>NoUpload</t>
+  </si>
+  <si>
+    <t>CAPEX_NUCLEAR_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-eligible nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>CAPEX_NUCLEAR_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-aligned nuclear activities (referred to in Sections 4.26, 4.27 and 4.28 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>CAPEX_GAS_ELIGIBLE_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-eligible fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>CAPEX_GAS_ALIGNED_PCT</t>
+  </si>
+  <si>
+    <t>Relative share of the CapEx that is associated with taxonomy-aligned fossil gas activities (referred to in Sections 4.29, 4.30 and 4.31 of Annexes I and II to Delegated Regulation (EU) 2021/2139)</t>
+  </si>
+  <si>
+    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentRevenueEligibleOrAlignedActivities]; EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentRevenueAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentRevenueNonAlignedActivities]</t>
+  </si>
+  <si>
+    <t>EuTaxonomyShare:[extendedEuTaxonomyEligibleOrAlignedActivitiesComponentCapexEligibleOrAlignedActivities]; EuTaxonomyShare:[extendedEuTaxonomyAlignedActivitiesComponentCapexAlignedActivities, extendedEuTaxonomyNonAlignedActivitiesComponentCapexNonAlignedActivities]</t>
   </si>
 </sst>
 </file>
@@ -870,7 +939,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Q58"/>
+  <dimension ref="A1:Q66"/>
   <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -1278,7 +1347,7 @@
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>61</v>
@@ -1310,7 +1379,7 @@
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>61</v>
@@ -1579,21 +1648,21 @@
       <c r="B26" t="s">
         <v>61</v>
       </c>
-      <c r="C26" t="s">
-        <v>102</v>
-      </c>
       <c r="D26" t="s">
-        <v>67</v>
+        <v>173</v>
       </c>
       <c r="E26" t="s">
-        <v>103</v>
+        <v>177</v>
       </c>
       <c r="F26" t="s">
-        <v>104</v>
+        <v>181</v>
       </c>
       <c r="G26" t="s">
         <v>70</v>
       </c>
+      <c r="H26" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="J26" t="s">
         <v>23</v>
       </c>
@@ -1602,6 +1671,9 @@
       </c>
       <c r="O26" t="s">
         <v>71</v>
+      </c>
+      <c r="Q26" s="3" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -1612,16 +1684,19 @@
         <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>174</v>
       </c>
       <c r="E27" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="F27" t="s">
-        <v>107</v>
+        <v>182</v>
       </c>
       <c r="G27" t="s">
-        <v>108</v>
+        <v>70</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J27" t="s">
         <v>23</v>
@@ -1633,7 +1708,7 @@
         <v>71</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -1641,19 +1716,22 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>62</v>
+        <v>175</v>
       </c>
       <c r="E28" t="s">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="F28" t="s">
-        <v>111</v>
+        <v>183</v>
       </c>
       <c r="G28" t="s">
-        <v>65</v>
+        <v>70</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J28" t="s">
         <v>23</v>
@@ -1663,6 +1741,9 @@
       </c>
       <c r="O28" t="s">
         <v>71</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -1670,23 +1751,23 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>67</v>
+        <v>176</v>
       </c>
       <c r="E29" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="F29" t="s">
-        <v>113</v>
+        <v>184</v>
       </c>
       <c r="G29" t="s">
         <v>70</v>
       </c>
+      <c r="H29" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="J29" t="s">
         <v>23</v>
       </c>
@@ -1695,29 +1776,32 @@
       </c>
       <c r="O29" t="s">
         <v>71</v>
+      </c>
+      <c r="Q29" s="3" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="D30" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E30" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="F30" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G30" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J30" t="s">
         <v>23</v>
@@ -1731,25 +1815,22 @@
     </row>
     <row r="31" spans="1:17">
       <c r="A31" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>109</v>
-      </c>
-      <c r="C31" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="E31" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="F31" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="G31" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="J31" t="s">
         <v>23</v>
@@ -1759,6 +1840,9 @@
       </c>
       <c r="O31" t="s">
         <v>71</v>
+      </c>
+      <c r="Q31" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -1769,16 +1853,16 @@
         <v>109</v>
       </c>
       <c r="D32" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E32" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="G32" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J32" t="s">
         <v>23</v>
@@ -1797,14 +1881,17 @@
       <c r="B33" t="s">
         <v>109</v>
       </c>
+      <c r="C33" t="s">
+        <v>66</v>
+      </c>
       <c r="D33" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="E33" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="F33" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="G33" t="s">
         <v>70</v>
@@ -1826,17 +1913,20 @@
       <c r="B34" t="s">
         <v>109</v>
       </c>
+      <c r="C34" t="s">
+        <v>72</v>
+      </c>
       <c r="D34" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="E34" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="G34" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J34" t="s">
         <v>23</v>
@@ -1855,14 +1945,17 @@
       <c r="B35" t="s">
         <v>109</v>
       </c>
+      <c r="C35" t="s">
+        <v>72</v>
+      </c>
       <c r="D35" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="E35" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="F35" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="G35" t="s">
         <v>70</v>
@@ -1885,13 +1978,13 @@
         <v>109</v>
       </c>
       <c r="D36" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E36" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="F36" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="G36" t="s">
         <v>70</v>
@@ -1914,13 +2007,13 @@
         <v>109</v>
       </c>
       <c r="D37" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E37" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F37" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="G37" t="s">
         <v>70</v>
@@ -1943,13 +2036,13 @@
         <v>109</v>
       </c>
       <c r="D38" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="E38" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="F38" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="G38" t="s">
         <v>70</v>
@@ -1972,13 +2065,13 @@
         <v>109</v>
       </c>
       <c r="D39" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="E39" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="F39" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="G39" t="s">
         <v>70</v>
@@ -2000,17 +2093,14 @@
       <c r="B40" t="s">
         <v>109</v>
       </c>
-      <c r="C40" t="s">
-        <v>102</v>
-      </c>
       <c r="D40" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="F40" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="G40" t="s">
         <v>70</v>
@@ -2033,16 +2123,16 @@
         <v>109</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="E41" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="G41" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="J41" t="s">
         <v>23</v>
@@ -2052,9 +2142,6 @@
       </c>
       <c r="O41" t="s">
         <v>71</v>
-      </c>
-      <c r="Q41" s="3" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:17">
@@ -2062,19 +2149,19 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D42" t="s">
-        <v>62</v>
+        <v>96</v>
       </c>
       <c r="E42" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="F42" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="G42" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J42" t="s">
         <v>23</v>
@@ -2091,19 +2178,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>138</v>
-      </c>
-      <c r="C43" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="D43" t="s">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="E43" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="F43" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="G43" t="s">
         <v>70</v>
@@ -2120,25 +2204,25 @@
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>138</v>
-      </c>
-      <c r="C44" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="D44" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="E44" t="s">
-        <v>143</v>
+        <v>186</v>
       </c>
       <c r="F44" t="s">
-        <v>144</v>
-      </c>
-      <c r="G44" t="s">
-        <v>65</v>
+        <v>187</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J44" t="s">
         <v>23</v>
@@ -2148,29 +2232,32 @@
       </c>
       <c r="O44" t="s">
         <v>71</v>
+      </c>
+      <c r="Q44" s="3" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:17">
       <c r="A45" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>138</v>
-      </c>
-      <c r="C45" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="D45" t="s">
-        <v>67</v>
+        <v>174</v>
       </c>
       <c r="E45" t="s">
-        <v>145</v>
+        <v>188</v>
       </c>
       <c r="F45" t="s">
-        <v>146</v>
-      </c>
-      <c r="G45" t="s">
-        <v>70</v>
+        <v>189</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J45" t="s">
         <v>23</v>
@@ -2180,6 +2267,9 @@
       </c>
       <c r="O45" t="s">
         <v>71</v>
+      </c>
+      <c r="Q45" s="3" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="46" spans="1:17">
@@ -2187,19 +2277,22 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D46" t="s">
-        <v>78</v>
+        <v>175</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>190</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
-      </c>
-      <c r="G46" t="s">
-        <v>70</v>
+        <v>191</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J46" t="s">
         <v>23</v>
@@ -2209,6 +2302,9 @@
       </c>
       <c r="O46" t="s">
         <v>71</v>
+      </c>
+      <c r="Q46" s="3" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:17">
@@ -2216,19 +2312,22 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D47" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
       <c r="E47" t="s">
-        <v>149</v>
+        <v>192</v>
       </c>
       <c r="F47" t="s">
-        <v>150</v>
-      </c>
-      <c r="G47" t="s">
-        <v>70</v>
+        <v>193</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="J47" t="s">
         <v>23</v>
@@ -2238,6 +2337,9 @@
       </c>
       <c r="O47" t="s">
         <v>71</v>
+      </c>
+      <c r="Q47" s="3" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:17">
@@ -2245,16 +2347,19 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>138</v>
+        <v>109</v>
+      </c>
+      <c r="C48" t="s">
+        <v>102</v>
       </c>
       <c r="D48" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="E48" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="F48" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="G48" t="s">
         <v>70</v>
@@ -2274,19 +2379,19 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D49" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="E49" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="F49" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="G49" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="J49" t="s">
         <v>23</v>
@@ -2296,6 +2401,9 @@
       </c>
       <c r="O49" t="s">
         <v>71</v>
+      </c>
+      <c r="Q49" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="50" spans="1:17">
@@ -2306,16 +2414,16 @@
         <v>138</v>
       </c>
       <c r="D50" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E50" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="F50" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="G50" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J50" t="s">
         <v>23</v>
@@ -2334,14 +2442,17 @@
       <c r="B51" t="s">
         <v>138</v>
       </c>
+      <c r="C51" t="s">
+        <v>66</v>
+      </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="E51" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="F51" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="G51" t="s">
         <v>70</v>
@@ -2363,17 +2474,20 @@
       <c r="B52" t="s">
         <v>138</v>
       </c>
+      <c r="C52" t="s">
+        <v>72</v>
+      </c>
       <c r="D52" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E52" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="F52" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="G52" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J52" t="s">
         <v>23</v>
@@ -2392,14 +2506,17 @@
       <c r="B53" t="s">
         <v>138</v>
       </c>
+      <c r="C53" t="s">
+        <v>72</v>
+      </c>
       <c r="D53" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="E53" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="F53" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="G53" t="s">
         <v>70</v>
@@ -2421,17 +2538,14 @@
       <c r="B54" t="s">
         <v>138</v>
       </c>
-      <c r="C54" t="s">
-        <v>102</v>
-      </c>
       <c r="D54" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E54" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="F54" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="G54" t="s">
         <v>70</v>
@@ -2454,38 +2568,273 @@
         <v>138</v>
       </c>
       <c r="D55" t="s">
+        <v>81</v>
+      </c>
+      <c r="E55" t="s">
+        <v>149</v>
+      </c>
+      <c r="F55" t="s">
+        <v>150</v>
+      </c>
+      <c r="G55" t="s">
+        <v>70</v>
+      </c>
+      <c r="J55" t="s">
+        <v>23</v>
+      </c>
+      <c r="N55" t="s">
+        <v>71</v>
+      </c>
+      <c r="O55" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
+      <c r="A56" s="2">
+        <v>54</v>
+      </c>
+      <c r="B56" t="s">
+        <v>138</v>
+      </c>
+      <c r="D56" t="s">
+        <v>84</v>
+      </c>
+      <c r="E56" t="s">
+        <v>151</v>
+      </c>
+      <c r="F56" t="s">
+        <v>152</v>
+      </c>
+      <c r="G56" t="s">
+        <v>70</v>
+      </c>
+      <c r="J56" t="s">
+        <v>23</v>
+      </c>
+      <c r="N56" t="s">
+        <v>71</v>
+      </c>
+      <c r="O56" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17">
+      <c r="A57" s="2">
+        <v>55</v>
+      </c>
+      <c r="B57" t="s">
+        <v>138</v>
+      </c>
+      <c r="D57" t="s">
+        <v>87</v>
+      </c>
+      <c r="E57" t="s">
+        <v>153</v>
+      </c>
+      <c r="F57" t="s">
+        <v>154</v>
+      </c>
+      <c r="G57" t="s">
+        <v>70</v>
+      </c>
+      <c r="J57" t="s">
+        <v>23</v>
+      </c>
+      <c r="N57" t="s">
+        <v>71</v>
+      </c>
+      <c r="O57" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17">
+      <c r="A58" s="2">
+        <v>56</v>
+      </c>
+      <c r="B58" t="s">
+        <v>138</v>
+      </c>
+      <c r="D58" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" t="s">
+        <v>155</v>
+      </c>
+      <c r="F58" t="s">
+        <v>156</v>
+      </c>
+      <c r="G58" t="s">
+        <v>70</v>
+      </c>
+      <c r="J58" t="s">
+        <v>23</v>
+      </c>
+      <c r="N58" t="s">
+        <v>71</v>
+      </c>
+      <c r="O58" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17">
+      <c r="A59" s="2">
+        <v>57</v>
+      </c>
+      <c r="B59" t="s">
+        <v>138</v>
+      </c>
+      <c r="D59" t="s">
+        <v>93</v>
+      </c>
+      <c r="E59" t="s">
+        <v>157</v>
+      </c>
+      <c r="F59" t="s">
+        <v>158</v>
+      </c>
+      <c r="G59" t="s">
+        <v>70</v>
+      </c>
+      <c r="J59" t="s">
+        <v>23</v>
+      </c>
+      <c r="N59" t="s">
+        <v>71</v>
+      </c>
+      <c r="O59" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17">
+      <c r="A60" s="2">
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>138</v>
+      </c>
+      <c r="D60" t="s">
+        <v>96</v>
+      </c>
+      <c r="E60" t="s">
+        <v>159</v>
+      </c>
+      <c r="F60" t="s">
+        <v>160</v>
+      </c>
+      <c r="G60" t="s">
+        <v>70</v>
+      </c>
+      <c r="J60" t="s">
+        <v>23</v>
+      </c>
+      <c r="N60" t="s">
+        <v>71</v>
+      </c>
+      <c r="O60" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17">
+      <c r="A61" s="2">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>138</v>
+      </c>
+      <c r="D61" t="s">
+        <v>99</v>
+      </c>
+      <c r="E61" t="s">
+        <v>161</v>
+      </c>
+      <c r="F61" t="s">
+        <v>162</v>
+      </c>
+      <c r="G61" t="s">
+        <v>70</v>
+      </c>
+      <c r="J61" t="s">
+        <v>23</v>
+      </c>
+      <c r="N61" t="s">
+        <v>71</v>
+      </c>
+      <c r="O61" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17">
+      <c r="A62" s="2">
+        <v>60</v>
+      </c>
+      <c r="B62" t="s">
+        <v>138</v>
+      </c>
+      <c r="C62" t="s">
+        <v>102</v>
+      </c>
+      <c r="D62" t="s">
+        <v>67</v>
+      </c>
+      <c r="E62" t="s">
+        <v>163</v>
+      </c>
+      <c r="F62" t="s">
+        <v>164</v>
+      </c>
+      <c r="G62" t="s">
+        <v>70</v>
+      </c>
+      <c r="J62" t="s">
+        <v>23</v>
+      </c>
+      <c r="N62" t="s">
+        <v>71</v>
+      </c>
+      <c r="O62" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17">
+      <c r="A63" s="2">
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>138</v>
+      </c>
+      <c r="D63" t="s">
         <v>105</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E63" t="s">
         <v>165</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F63" t="s">
         <v>166</v>
       </c>
-      <c r="G55" t="s">
+      <c r="G63" t="s">
         <v>108</v>
       </c>
-      <c r="J55" t="s">
-        <v>23</v>
-      </c>
-      <c r="N55" t="s">
-        <v>71</v>
-      </c>
-      <c r="O55" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q55" s="5" t="s">
+      <c r="J63" t="s">
+        <v>23</v>
+      </c>
+      <c r="N63" t="s">
+        <v>71</v>
+      </c>
+      <c r="O63" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q63" s="5" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="56" spans="1:17">
-      <c r="A56" s="2"/>
-    </row>
-    <row r="57" spans="1:17">
-      <c r="A57" s="2"/>
-    </row>
-    <row r="58" spans="1:17">
-      <c r="A58" s="2"/>
+    <row r="64" spans="1:17">
+      <c r="A64" s="2"/>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="2"/>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>